<commit_message>
[feat/ASP-2692-Vietnam-Report-M4B3] Tweaks for development
</commit_message>
<xml_diff>
--- a/api/templates/geneXpert_M4B3_biological_products/en.xlsx
+++ b/api/templates/geneXpert_M4B3_biological_products/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\ahernandez\repos\aspect\api\templates\geneXpert_M4B3_biological_products\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42E58DBA-0911-4047-A0D7-B301F1BC2A7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84ADB67B-4178-4456-B93E-31997C0D800D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{24D7A4EE-8982-41AB-893B-67BF3AF2DD3B}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="M4B3.Biological product" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'M4B3.Biological product'!$A$1:$O$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'M4B3.Biological product'!$A$1:$O$26</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="55">
   <si>
     <r>
       <t xml:space="preserve">                            MINISTRY OF HEALTH                                                                                                         </t>
@@ -63,9 +63,6 @@
     <t>REPORT ON USE OF XPERT BIOLOGICAL PRODUCTS</t>
   </si>
   <si>
-    <t xml:space="preserve">Month        year </t>
-  </si>
-  <si>
     <t xml:space="preserve">Laboratory: </t>
   </si>
   <si>
@@ -75,9 +72,6 @@
     <t xml:space="preserve">Province: </t>
   </si>
   <si>
-    <t xml:space="preserve">Tel phone:               Email: </t>
-  </si>
-  <si>
     <t>No.</t>
   </si>
   <si>
@@ -147,9 +141,6 @@
     <t>(Sign, full name)</t>
   </si>
   <si>
-    <t>&lt;Lgas&gt;</t>
-  </si>
-  <si>
     <t>&lt;States&gt;</t>
   </si>
   <si>
@@ -202,13 +193,34 @@
   </si>
   <si>
     <t>&lt;receiveTo&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Sites&gt;</t>
+  </si>
+  <si>
+    <t>Tel phone:</t>
+  </si>
+  <si>
+    <t>&lt;UserMobilePhone&gt;</t>
+  </si>
+  <si>
+    <t>&lt;UserFullName&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email :   </t>
+  </si>
+  <si>
+    <t>&lt;UserEmail&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Dates&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -243,14 +255,6 @@
     </font>
     <font>
       <sz val="13"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -356,6 +360,33 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="13"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -542,7 +573,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -568,40 +599,36 @@
       <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="4"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" indent="4"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="4"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
@@ -610,42 +637,137 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -653,91 +775,16 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="22" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1055,7 +1102,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2C291B8-9532-4480-AFE4-4C26C045E395}">
-  <dimension ref="A1:Q28"/>
+  <dimension ref="A1:Q27"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.6640625" style="3" customWidth="1"/>
@@ -2045,95 +2092,103 @@
       <c r="D3" s="6"/>
     </row>
     <row r="4" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
-      <c r="J4" s="31"/>
-      <c r="K4" s="31"/>
-      <c r="L4" s="31"/>
-      <c r="M4" s="31"/>
-      <c r="N4" s="31"/>
-      <c r="O4" s="31"/>
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54"/>
+      <c r="K4" s="54"/>
+      <c r="L4" s="54"/>
+      <c r="M4" s="54"/>
+      <c r="N4" s="54"/>
+      <c r="O4" s="54"/>
       <c r="P4" s="7"/>
     </row>
-    <row r="5" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="32" t="s">
+    <row r="5" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="57" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="57"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="57"/>
+      <c r="I5" s="57"/>
+      <c r="J5" s="57"/>
+      <c r="K5" s="57"/>
+      <c r="L5" s="57"/>
+      <c r="M5" s="57"/>
+      <c r="N5" s="57"/>
+      <c r="O5" s="57"/>
+      <c r="P5" s="8"/>
+    </row>
+    <row r="6" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="32"/>
-      <c r="K5" s="32"/>
-      <c r="L5" s="32"/>
-      <c r="M5" s="32"/>
-      <c r="N5" s="32"/>
-      <c r="O5" s="32"/>
-      <c r="P5" s="8"/>
-    </row>
-    <row r="6" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="24" t="s">
+      <c r="B6" s="22"/>
+      <c r="C6" s="55" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="23" t="s">
+      <c r="H6" s="56" t="s">
+        <v>51</v>
+      </c>
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
+      <c r="K6" s="56"/>
+      <c r="L6" s="56"/>
+      <c r="M6" s="56"/>
+      <c r="N6" s="56"/>
+      <c r="O6" s="56"/>
+      <c r="P6" s="10"/>
+    </row>
+    <row r="7" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
-      <c r="N6" s="23"/>
-      <c r="O6" s="23"/>
-      <c r="P6" s="10"/>
-    </row>
-    <row r="7" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="55" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="55"/>
+      <c r="E7" s="55"/>
       <c r="F7" s="9"/>
-      <c r="G7" s="33" t="s">
-        <v>8</v>
-      </c>
-      <c r="H7" s="33"/>
-      <c r="I7" s="33"/>
-      <c r="J7" s="33"/>
-      <c r="K7" s="33"/>
-      <c r="L7" s="33"/>
-      <c r="M7" s="33"/>
-      <c r="N7" s="33"/>
-      <c r="O7" s="33"/>
+      <c r="G7" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" s="56" t="s">
+        <v>50</v>
+      </c>
+      <c r="I7" s="56"/>
+      <c r="J7" s="56"/>
+      <c r="K7" s="44" t="s">
+        <v>52</v>
+      </c>
+      <c r="L7" s="56" t="s">
+        <v>53</v>
+      </c>
+      <c r="M7" s="56"/>
+      <c r="N7" s="56"/>
+      <c r="O7" s="56"/>
     </row>
     <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B8" s="9">
         <v>2</v>
@@ -2154,271 +2209,288 @@
       <c r="P8" s="11"/>
     </row>
     <row r="9" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="51" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="51" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="36" t="s">
+      <c r="D9" s="51" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="37" t="s">
+      <c r="E9" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="36" t="s">
+      <c r="F9" s="51" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="36" t="s">
+      <c r="G9" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="36" t="s">
+      <c r="H9" s="51"/>
+      <c r="I9" s="51"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="51"/>
+      <c r="L9" s="51"/>
+      <c r="M9" s="51"/>
+      <c r="N9" s="51"/>
+      <c r="O9" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="36" t="s">
+      <c r="P9" s="10"/>
+    </row>
+    <row r="10" spans="1:17" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="51"/>
+      <c r="B10" s="51"/>
+      <c r="C10" s="53"/>
+      <c r="D10" s="51"/>
+      <c r="E10" s="51"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="36"/>
-      <c r="I9" s="36"/>
-      <c r="J9" s="36"/>
-      <c r="K9" s="36"/>
-      <c r="L9" s="36"/>
-      <c r="M9" s="36"/>
-      <c r="N9" s="36"/>
-      <c r="O9" s="36" t="s">
+      <c r="H10" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="P9" s="10"/>
-    </row>
-    <row r="10" spans="1:17" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="36"/>
-      <c r="B10" s="36"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="36"/>
-      <c r="G10" s="26" t="s">
+      <c r="I10" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="26" t="s">
+      <c r="J10" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="K10" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="L10" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="M10" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="N10" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="K10" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="L10" s="26" t="s">
-        <v>40</v>
-      </c>
-      <c r="M10" s="26" t="s">
-        <v>45</v>
-      </c>
-      <c r="N10" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="O10" s="36"/>
+      <c r="O10" s="51"/>
       <c r="P10" s="10"/>
     </row>
     <row r="11" spans="1:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B11" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="13" t="s">
-        <v>38</v>
-      </c>
       <c r="D11" s="13" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="F11" s="30" t="s">
-        <v>47</v>
-      </c>
-      <c r="G11" s="39" t="e">
+        <v>31</v>
+      </c>
+      <c r="F11" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" s="29" t="e">
         <f>O11+H11+I11-SUM(J11:N11)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="H11" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="I11" s="40" t="s">
-        <v>49</v>
-      </c>
-      <c r="J11" s="28" t="s">
-        <v>50</v>
-      </c>
-      <c r="K11" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="L11" s="28" t="s">
+      <c r="H11" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="I11" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="J11" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="K11" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="L11" s="26" t="s">
+        <v>40</v>
+      </c>
+      <c r="M11" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="M11" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="N11" s="28" t="s">
-        <v>44</v>
-      </c>
-      <c r="O11" s="15" t="s">
-        <v>35</v>
+      <c r="N11" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="O11" s="14" t="s">
+        <v>32</v>
       </c>
       <c r="P11" s="7"/>
     </row>
-    <row r="12" spans="1:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="41" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="42"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="42"/>
-      <c r="E13" s="42"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="27" t="e">
+    <row r="12" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="25" t="e">
         <f>SUM(G$11:G11)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="H13" s="27">
+      <c r="H12" s="25">
         <f>SUM(H$11:H11)</f>
         <v>0</v>
       </c>
-      <c r="I13" s="27">
+      <c r="I12" s="25">
         <f>SUM(I$11:I11)</f>
         <v>0</v>
       </c>
-      <c r="J13" s="27">
+      <c r="J12" s="25">
         <f>SUM(J$11:J11)</f>
         <v>0</v>
       </c>
-      <c r="K13" s="27">
+      <c r="K12" s="25">
         <f>SUM(K$11:K11)</f>
         <v>0</v>
       </c>
-      <c r="L13" s="27">
+      <c r="L12" s="25">
         <f>SUM(L$11:L11)</f>
         <v>0</v>
       </c>
-      <c r="M13" s="27">
+      <c r="M12" s="25">
         <f>SUM(M$11:M11)</f>
         <v>0</v>
       </c>
-      <c r="N13" s="27">
+      <c r="N12" s="25">
         <f>SUM(N$11:N11)</f>
         <v>0</v>
       </c>
-      <c r="O13" s="27">
+      <c r="O12" s="25">
         <f>SUM(O$11:O11)</f>
         <v>0</v>
       </c>
+      <c r="P12" s="7"/>
+    </row>
+    <row r="13" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
       <c r="P13" s="7"/>
     </row>
-    <row r="14" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="7"/>
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
+    <row r="14" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="35"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="E14" s="34"/>
+      <c r="F14" s="45"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="46"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="15"/>
+      <c r="L14" s="15"/>
+      <c r="M14" s="15"/>
+      <c r="N14" s="15"/>
+      <c r="O14" s="15"/>
       <c r="P14" s="7"/>
     </row>
     <row r="15" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="45"/>
-      <c r="B15" s="46"/>
-      <c r="C15" s="47"/>
-      <c r="D15" s="44" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15" s="44"/>
-      <c r="F15" s="44"/>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="14"/>
+      <c r="A15" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="39"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="46"/>
+      <c r="I15" s="48"/>
       <c r="J15" s="16"/>
       <c r="K15" s="16"/>
       <c r="L15" s="16"/>
       <c r="M15" s="16"/>
-      <c r="N15" s="16"/>
-      <c r="O15" s="16"/>
+      <c r="N15" s="15"/>
+      <c r="O15" s="15"/>
       <c r="P15" s="7"/>
+      <c r="Q15" s="16"/>
     </row>
     <row r="16" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="48" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="49"/>
-      <c r="C16" s="50"/>
-      <c r="D16" s="44" t="s">
+      <c r="A16" s="41"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="45"/>
+      <c r="H16" s="46"/>
+      <c r="I16" s="48"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="15"/>
+      <c r="O16" s="15"/>
+      <c r="P16" s="7"/>
+    </row>
+    <row r="17" spans="1:16" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="15"/>
+      <c r="L17" s="15"/>
+      <c r="M17" s="15"/>
+      <c r="N17" s="15"/>
+      <c r="O17" s="15"/>
+      <c r="P17" s="7"/>
+    </row>
+    <row r="18" spans="1:16" s="17" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G18" s="15"/>
+      <c r="I18" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="44"/>
-      <c r="F16" s="44"/>
-      <c r="G16" s="44"/>
-      <c r="H16" s="44"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
-      <c r="M16" s="18"/>
-      <c r="N16" s="16"/>
-      <c r="O16" s="16"/>
-      <c r="P16" s="7"/>
-      <c r="Q16" s="18"/>
-    </row>
-    <row r="17" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="51"/>
-      <c r="B17" s="52"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="44" t="s">
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18"/>
+      <c r="M18" s="18"/>
+    </row>
+    <row r="19" spans="1:16" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="49" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="44"/>
-      <c r="F17" s="44"/>
-      <c r="G17" s="44"/>
-      <c r="H17" s="44"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
-      <c r="L17" s="18"/>
-      <c r="M17" s="18"/>
-      <c r="N17" s="16"/>
-      <c r="O17" s="16"/>
-      <c r="P17" s="7"/>
-    </row>
-    <row r="18" spans="1:16" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="16"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="16"/>
-      <c r="O18" s="16"/>
-      <c r="P18" s="7"/>
-    </row>
-    <row r="19" spans="1:16" s="19" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="G19" s="16"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="19"/>
       <c r="I19" s="20" t="s">
         <v>27</v>
       </c>
@@ -2427,84 +2499,70 @@
       <c r="L19" s="20"/>
       <c r="M19" s="20"/>
     </row>
-    <row r="20" spans="1:16" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="34" t="s">
+    <row r="20" spans="1:16" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="C20" s="34"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="22" t="s">
+      <c r="C20" s="50"/>
+      <c r="G20" s="15"/>
+      <c r="I20" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="J20" s="22"/>
-      <c r="K20" s="22"/>
-      <c r="L20" s="22"/>
-      <c r="M20" s="22"/>
-    </row>
-    <row r="21" spans="1:16" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="35" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="35"/>
-      <c r="G21" s="16"/>
-      <c r="I21" s="35" t="s">
-        <v>31</v>
-      </c>
-      <c r="J21" s="35"/>
-      <c r="K21" s="25"/>
-      <c r="L21" s="25"/>
-      <c r="M21" s="25"/>
-    </row>
-    <row r="22" spans="1:16" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="G22" s="16"/>
+      <c r="J20" s="50"/>
+      <c r="K20" s="23"/>
+      <c r="L20" s="23"/>
+      <c r="M20" s="23"/>
+    </row>
+    <row r="21" spans="1:16" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="G21" s="15"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
+      <c r="L22" s="27"/>
+      <c r="M22" s="27"/>
+      <c r="N22" s="27"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="F23" s="29"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="29"/>
-      <c r="I23" s="29"/>
-      <c r="J23" s="29"/>
-      <c r="K23" s="29"/>
-      <c r="L23" s="29"/>
-      <c r="M23" s="29"/>
-      <c r="N23" s="29"/>
+      <c r="E23" s="27"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="E24" s="29"/>
+      <c r="E24" s="27"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="E25" s="29"/>
+      <c r="E25" s="27"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="E26" s="29"/>
+      <c r="E26" s="27"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="E27" s="29"/>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="E28" s="29"/>
+      <c r="E27" s="27"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
-  <mergeCells count="14">
+  <mergeCells count="18">
+    <mergeCell ref="A4:O4"/>
+    <mergeCell ref="A5:O5"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="H6:O6"/>
+    <mergeCell ref="L7:O7"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="G9:N9"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
     <mergeCell ref="D9:D10"/>
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="F9:F10"/>
-    <mergeCell ref="A4:O4"/>
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="G7:O7"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="G9:N9"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.25" top="0.5" bottom="0.25" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
[feat/ASP-2692-Vietnam-Report-M4B3] Modified the zoom in xlsx to better adapt to the likely width of the user's screen.
</commit_message>
<xml_diff>
--- a/api/templates/geneXpert_M4B3_biological_products/en.xlsx
+++ b/api/templates/geneXpert_M4B3_biological_products/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\ahernandez\repos\aspect\api\templates\geneXpert_M4B3_biological_products\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FE604BD-FE6E-4162-B680-86F51754F61A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A1EF022-F848-4434-8E91-7609807316E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{24D7A4EE-8982-41AB-893B-67BF3AF2DD3B}"/>
   </bookViews>
@@ -781,48 +781,48 @@
     <xf numFmtId="3" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="5"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="5"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -2102,26 +2102,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="58" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
       <c r="F1" s="1"/>
       <c r="P1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="58" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
       <c r="F2" s="1"/>
       <c r="G2" s="4"/>
     </row>
@@ -2133,45 +2133,45 @@
       <c r="E3" s="5"/>
     </row>
     <row r="4" spans="1:18" ht="24" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="53"/>
-      <c r="C4" s="53"/>
-      <c r="D4" s="53"/>
-      <c r="E4" s="53"/>
-      <c r="F4" s="53"/>
-      <c r="G4" s="53"/>
-      <c r="H4" s="53"/>
-      <c r="I4" s="53"/>
-      <c r="J4" s="53"/>
-      <c r="K4" s="53"/>
-      <c r="L4" s="53"/>
-      <c r="M4" s="53"/>
-      <c r="N4" s="53"/>
-      <c r="O4" s="53"/>
-      <c r="P4" s="53"/>
+      <c r="B4" s="52"/>
+      <c r="C4" s="52"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="52"/>
+      <c r="H4" s="52"/>
+      <c r="I4" s="52"/>
+      <c r="J4" s="52"/>
+      <c r="K4" s="52"/>
+      <c r="L4" s="52"/>
+      <c r="M4" s="52"/>
+      <c r="N4" s="52"/>
+      <c r="O4" s="52"/>
+      <c r="P4" s="52"/>
       <c r="Q4" s="6"/>
     </row>
     <row r="5" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="54" t="s">
+      <c r="A5" s="53" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
-      <c r="H5" s="54"/>
-      <c r="I5" s="54"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="54"/>
-      <c r="L5" s="54"/>
-      <c r="M5" s="54"/>
-      <c r="N5" s="54"/>
-      <c r="O5" s="54"/>
-      <c r="P5" s="54"/>
+      <c r="B5" s="53"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="53"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53"/>
+      <c r="G5" s="53"/>
+      <c r="H5" s="53"/>
+      <c r="I5" s="53"/>
+      <c r="J5" s="53"/>
+      <c r="K5" s="53"/>
+      <c r="L5" s="53"/>
+      <c r="M5" s="53"/>
+      <c r="N5" s="53"/>
+      <c r="O5" s="53"/>
+      <c r="P5" s="53"/>
       <c r="Q5" s="7"/>
     </row>
     <row r="6" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2179,26 +2179,26 @@
         <v>2</v>
       </c>
       <c r="B6" s="20"/>
-      <c r="C6" s="55" t="s">
+      <c r="C6" s="54" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="55"/>
-      <c r="E6" s="55"/>
-      <c r="F6" s="55"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
       <c r="G6" s="8"/>
       <c r="H6" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="I6" s="56" t="s">
+      <c r="I6" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="J6" s="56"/>
-      <c r="K6" s="56"/>
-      <c r="L6" s="56"/>
-      <c r="M6" s="56"/>
-      <c r="N6" s="56"/>
-      <c r="O6" s="56"/>
-      <c r="P6" s="56"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="55"/>
+      <c r="L6" s="55"/>
+      <c r="M6" s="55"/>
+      <c r="N6" s="55"/>
+      <c r="O6" s="55"/>
+      <c r="P6" s="55"/>
       <c r="Q6" s="9"/>
     </row>
     <row r="7" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2206,30 +2206,30 @@
         <v>4</v>
       </c>
       <c r="B7" s="20"/>
-      <c r="C7" s="55" t="s">
+      <c r="C7" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55"/>
-      <c r="F7" s="55"/>
+      <c r="D7" s="54"/>
+      <c r="E7" s="54"/>
+      <c r="F7" s="54"/>
       <c r="G7" s="8"/>
       <c r="H7" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="I7" s="56" t="s">
+      <c r="I7" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="J7" s="56"/>
-      <c r="K7" s="56"/>
+      <c r="J7" s="55"/>
+      <c r="K7" s="55"/>
       <c r="L7" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="M7" s="56" t="s">
+      <c r="M7" s="55" t="s">
         <v>48</v>
       </c>
-      <c r="N7" s="56"/>
-      <c r="O7" s="56"/>
-      <c r="P7" s="56"/>
+      <c r="N7" s="55"/>
+      <c r="O7" s="55"/>
+      <c r="P7" s="55"/>
     </row>
     <row r="8" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
@@ -2255,50 +2255,50 @@
       <c r="Q8" s="10"/>
     </row>
     <row r="9" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="49" t="s">
+      <c r="A9" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="49" t="s">
+      <c r="B9" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="57" t="s">
+      <c r="C9" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="57" t="s">
+      <c r="D9" s="56" t="s">
         <v>61</v>
       </c>
-      <c r="E9" s="49" t="s">
+      <c r="E9" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="49" t="s">
+      <c r="F9" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="49" t="s">
+      <c r="G9" s="51" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="49" t="s">
+      <c r="H9" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="49"/>
-      <c r="J9" s="49"/>
-      <c r="K9" s="49"/>
-      <c r="L9" s="49"/>
-      <c r="M9" s="49"/>
-      <c r="N9" s="49"/>
-      <c r="O9" s="49"/>
-      <c r="P9" s="49" t="s">
+      <c r="I9" s="51"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="51"/>
+      <c r="L9" s="51"/>
+      <c r="M9" s="51"/>
+      <c r="N9" s="51"/>
+      <c r="O9" s="51"/>
+      <c r="P9" s="51" t="s">
         <v>12</v>
       </c>
       <c r="Q9" s="9"/>
     </row>
     <row r="10" spans="1:18" ht="51.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="49"/>
-      <c r="B10" s="49"/>
-      <c r="C10" s="58"/>
-      <c r="D10" s="58"/>
-      <c r="E10" s="49"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="49"/>
+      <c r="A10" s="51"/>
+      <c r="B10" s="51"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="51"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="51"/>
       <c r="H10" s="22" t="s">
         <v>13</v>
       </c>
@@ -2323,7 +2323,7 @@
       <c r="O10" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="49"/>
+      <c r="P10" s="51"/>
       <c r="Q10" s="9"/>
     </row>
     <row r="11" spans="1:18" ht="26.1" customHeight="1" x14ac:dyDescent="0.3">
@@ -2528,7 +2528,7 @@
     </row>
     <row r="18" spans="1:17" s="15" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H18" s="13"/>
-      <c r="J18" s="59" t="s">
+      <c r="J18" s="49" t="s">
         <v>57</v>
       </c>
       <c r="K18" s="16"/>
@@ -2537,10 +2537,10 @@
       <c r="N18" s="16"/>
     </row>
     <row r="19" spans="1:17" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="51" t="s">
+      <c r="B19" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="51"/>
+      <c r="C19" s="59"/>
       <c r="D19" s="41"/>
       <c r="E19" s="17"/>
       <c r="F19" s="17"/>
@@ -2556,16 +2556,16 @@
       <c r="N19" s="18"/>
     </row>
     <row r="20" spans="1:17" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="52" t="s">
+      <c r="B20" s="50" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="52"/>
+      <c r="C20" s="50"/>
       <c r="D20" s="42"/>
       <c r="H20" s="13"/>
-      <c r="J20" s="52" t="s">
+      <c r="J20" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="K20" s="52"/>
+      <c r="K20" s="50"/>
       <c r="L20" s="21"/>
       <c r="M20" s="21"/>
       <c r="N20" s="21"/>
@@ -2602,6 +2602,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="21">
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="J20:K20"/>
     <mergeCell ref="H9:O9"/>
@@ -2618,11 +2623,6 @@
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="D9:D10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="B19:C19"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.25" top="0.5" bottom="0.25" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>